<commit_message>
Add new email signature designs and logo assets for Jordan Scheftic
- Created two new HTML email signature designs: jordannew_design2.html and jordannew_design3.html
- Added SVG logos for LinkedIn and X (formerly Twitter)
- Developed a logo generator HTML page for SPSI logo variations
- Introduced SVG logos for X and X logo in black
- Updated existing email signature template for Jordan Scheftic with new design elements
</commit_message>
<xml_diff>
--- a/employees_spsi.xlsx
+++ b/employees_spsi.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jscheftic\SPSI Code\SPSI Signatures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0AC1D53-AFDD-4197-8F1D-0B35140A6237}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EB8AB29-59BA-42B1-AF16-D0560366432B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3030" yWindow="-14610" windowWidth="21600" windowHeight="12525" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-30" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="159">
   <si>
     <t>Name</t>
   </si>
@@ -124,9 +124,6 @@
     <t>Val Martinez</t>
   </si>
   <si>
-    <t>Ross Esenberg</t>
-  </si>
-  <si>
     <t>Accounts Receivable</t>
   </si>
   <si>
@@ -181,9 +178,6 @@
     <t>Admin</t>
   </si>
   <si>
-    <t>Director, Sales &amp; Service</t>
-  </si>
-  <si>
     <t>763-391-7390</t>
   </si>
   <si>
@@ -196,9 +190,6 @@
     <t>1035</t>
   </si>
   <si>
-    <t>1013</t>
-  </si>
-  <si>
     <t>1345</t>
   </si>
   <si>
@@ -331,9 +322,6 @@
     <t>763-255-1021</t>
   </si>
   <si>
-    <t>612-309-1660</t>
-  </si>
-  <si>
     <t>918-499-0018</t>
   </si>
   <si>
@@ -448,9 +436,6 @@
     <t>vmartinez@spsi.com</t>
   </si>
   <si>
-    <t>resenberg@spsi.com</t>
-  </si>
-  <si>
     <t>mbunde@spsi.com</t>
   </si>
   <si>
@@ -487,20 +472,41 @@
     <t>balvarez@spsi.com</t>
   </si>
   <si>
-    <t>Case Bartow</t>
-  </si>
-  <si>
     <t>Service &amp; Parts Manager</t>
   </si>
   <si>
     <t>Business System Solutions Integrator</t>
+  </si>
+  <si>
+    <t>Liz Beavers</t>
+  </si>
+  <si>
+    <t>Embroidery Consultant</t>
+  </si>
+  <si>
+    <t>254-931-1063</t>
+  </si>
+  <si>
+    <t>lbeavers@spsi.com</t>
+  </si>
+  <si>
+    <t>Mason McCann</t>
+  </si>
+  <si>
+    <t>651-261-3070</t>
+  </si>
+  <si>
+    <t>mmccann@spsicom</t>
+  </si>
+  <si>
+    <t>South Central Manager</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -538,6 +544,12 @@
     </font>
     <font>
       <sz val="9.5"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="14"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
@@ -594,7 +606,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -608,6 +620,7 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -936,13 +949,13 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>2</v>
@@ -963,28 +976,28 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F2" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G2" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="G2" s="3" t="s">
-        <v>55</v>
-      </c>
       <c r="H2" s="3" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="I2" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="J2" s="2"/>
     </row>
@@ -993,28 +1006,28 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="J3" s="2"/>
     </row>
@@ -1023,28 +1036,28 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G4" s="3">
         <v>1037</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="J4" s="2"/>
     </row>
@@ -1053,28 +1066,28 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D5" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="I5" t="s">
         <v>112</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="I5" t="s">
-        <v>116</v>
       </c>
       <c r="J5" s="2"/>
     </row>
@@ -1083,28 +1096,28 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E6" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="I6" t="s">
         <v>113</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="I6" t="s">
-        <v>117</v>
       </c>
       <c r="J6" s="2"/>
     </row>
@@ -1113,28 +1126,28 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="I7" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="J7" s="2"/>
     </row>
@@ -1143,28 +1156,28 @@
         <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="I8" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="J8" s="2"/>
     </row>
@@ -1173,28 +1186,28 @@
         <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="I9" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="J9" s="2"/>
     </row>
@@ -1203,28 +1216,28 @@
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="I10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="J10" s="2"/>
     </row>
@@ -1233,28 +1246,28 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="J11" s="2"/>
     </row>
@@ -1263,26 +1276,26 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G12" s="3"/>
       <c r="H12" s="3" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="I12" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="J12" s="2"/>
     </row>
@@ -1291,26 +1304,26 @@
         <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C13" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="E13" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="D13" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>115</v>
-      </c>
       <c r="F13" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H13" s="3"/>
       <c r="I13" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="J13" s="2"/>
     </row>
@@ -1319,28 +1332,28 @@
         <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="I14" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="J14" s="2"/>
     </row>
@@ -1349,28 +1362,28 @@
         <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="I15" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="J15" s="2"/>
     </row>
@@ -1379,28 +1392,28 @@
         <v>20</v>
       </c>
       <c r="B16" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="I16" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="J16" s="2"/>
     </row>
@@ -1409,28 +1422,28 @@
         <v>21</v>
       </c>
       <c r="B17" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="I17" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="J17" s="2"/>
     </row>
@@ -1439,26 +1452,26 @@
         <v>22</v>
       </c>
       <c r="B18" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G18" s="3"/>
       <c r="H18" s="3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="I18" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="J18" s="2"/>
     </row>
@@ -1467,26 +1480,26 @@
         <v>23</v>
       </c>
       <c r="B19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G19" s="3"/>
       <c r="H19" s="3" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="I19" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="J19" s="2"/>
     </row>
@@ -1495,28 +1508,28 @@
         <v>24</v>
       </c>
       <c r="B20" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="I20" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="J20" s="2"/>
     </row>
@@ -1525,26 +1538,26 @@
         <v>25</v>
       </c>
       <c r="B21" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G21" s="3"/>
       <c r="H21" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="J21" s="2"/>
     </row>
@@ -1553,28 +1566,28 @@
         <v>26</v>
       </c>
       <c r="B22" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="I22" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="J22" s="2"/>
     </row>
@@ -1583,28 +1596,28 @@
         <v>27</v>
       </c>
       <c r="B23" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="I23" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="J23" s="2"/>
     </row>
@@ -1613,58 +1626,58 @@
         <v>28</v>
       </c>
       <c r="B24" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="I24" s="4" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="J24" s="2"/>
     </row>
     <row r="25" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="B25" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="I25" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J25" s="2"/>
     </row>
@@ -1673,26 +1686,26 @@
         <v>29</v>
       </c>
       <c r="B26" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G26" s="3"/>
       <c r="H26" s="3" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="I26" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="J26" s="2"/>
     </row>
@@ -1701,28 +1714,28 @@
         <v>30</v>
       </c>
       <c r="B27" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="I27" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="J27" s="2"/>
     </row>
@@ -1731,28 +1744,28 @@
         <v>31</v>
       </c>
       <c r="B28" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="I28" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="J28" s="2"/>
     </row>
@@ -1761,28 +1774,28 @@
         <v>32</v>
       </c>
       <c r="B29" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="I29" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="J29" s="2"/>
     </row>
@@ -1790,29 +1803,22 @@
       <c r="A30" t="s">
         <v>33</v>
       </c>
-      <c r="B30" t="s">
-        <v>52</v>
-      </c>
       <c r="C30" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="G30" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="H30" s="3" t="s">
-        <v>102</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
       <c r="I30" t="s">
-        <v>141</v>
+        <v>100</v>
       </c>
       <c r="J30" s="2"/>
     </row>
@@ -1821,21 +1827,21 @@
         <v>34</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G31" s="3"/>
       <c r="H31" s="3"/>
       <c r="I31" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="J31" s="2"/>
     </row>
@@ -1844,149 +1850,155 @@
         <v>35</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G32" s="3"/>
       <c r="H32" s="3"/>
       <c r="I32" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="J32" s="2"/>
     </row>
-    <row r="33" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>36</v>
+        <v>141</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>158</v>
       </c>
       <c r="C33" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="E33" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="D33" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="E33" s="3" t="s">
-        <v>113</v>
-      </c>
       <c r="F33" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="G33" s="3"/>
-      <c r="H33" s="3"/>
-      <c r="I33" t="s">
-        <v>106</v>
-      </c>
-      <c r="J33" s="2"/>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+      <c r="H33" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="I33" s="5" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
+        <v>143</v>
+      </c>
+      <c r="B34" t="s">
+        <v>47</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G34">
+        <v>1008</v>
+      </c>
+      <c r="H34" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="I34" s="5" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>146</v>
       </c>
-      <c r="B34" t="s">
-        <v>44</v>
-      </c>
-      <c r="C34" s="3" t="s">
+      <c r="B35" t="s">
+        <v>47</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H35" t="s">
+        <v>147</v>
+      </c>
+      <c r="I35" s="5" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A36" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="E36" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="D34" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="E34" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="F34" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="H34" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="I34" s="5" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
-        <v>148</v>
-      </c>
-      <c r="B35" t="s">
-        <v>48</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="D35" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="E35" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="F35" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="G35">
-        <v>1008</v>
-      </c>
-      <c r="H35" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="I35" s="5" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>151</v>
-      </c>
-      <c r="B36" t="s">
-        <v>48</v>
-      </c>
-      <c r="C36" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="D36" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="E36" s="3" t="s">
-        <v>113</v>
-      </c>
       <c r="F36" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="H36" t="s">
-        <v>152</v>
+        <v>52</v>
+      </c>
+      <c r="H36" s="7" t="s">
+        <v>153</v>
       </c>
       <c r="I36" s="5" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
         <v>154</v>
       </c>
-      <c r="B37" t="s">
-        <v>45</v>
+    </row>
+    <row r="37" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A37" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>43</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="G37">
-        <v>1065</v>
+        <v>51</v>
+      </c>
+      <c r="H37" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="I37" s="5" t="s">
+        <v>157</v>
       </c>
     </row>
   </sheetData>
@@ -1998,9 +2010,11 @@
     <hyperlink ref="I21" r:id="rId3" xr:uid="{6AAED2F0-F8D8-4FF4-ACD1-C31F181977F0}"/>
     <hyperlink ref="I24" r:id="rId4" xr:uid="{D0ADFA12-4299-465B-9A7F-9CAD2594F893}"/>
     <hyperlink ref="I4" r:id="rId5" xr:uid="{D65B02A3-28F0-4EC6-A7A0-E462DF63F258}"/>
-    <hyperlink ref="I34" r:id="rId6" xr:uid="{44CB69C5-8668-4D15-9AC8-28BD0941640E}"/>
-    <hyperlink ref="I35" r:id="rId7" xr:uid="{455D0F10-5F93-4934-8480-A2ADB02ADB24}"/>
-    <hyperlink ref="I36" r:id="rId8" xr:uid="{809D9758-0FE4-4826-A9DB-D6860327E3A1}"/>
+    <hyperlink ref="I33" r:id="rId6" xr:uid="{44CB69C5-8668-4D15-9AC8-28BD0941640E}"/>
+    <hyperlink ref="I34" r:id="rId7" xr:uid="{455D0F10-5F93-4934-8480-A2ADB02ADB24}"/>
+    <hyperlink ref="I35" r:id="rId8" xr:uid="{809D9758-0FE4-4826-A9DB-D6860327E3A1}"/>
+    <hyperlink ref="I36" r:id="rId9" xr:uid="{D253A6F8-193A-4864-868D-36CAFD4E39CE}"/>
+    <hyperlink ref="I37" r:id="rId10" xr:uid="{648EABE6-7C55-467B-9A28-2D6546C6E22C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>